<commit_message>
Faz 1: cost engine with manual geometry input, reports, storage, UI
- Pure cost formulas (learning curve, operation time, labor, machine,
  ply material, consumables, autoclave share, overhead, price)
- Quote engine producing traceable CostLines with sources and library
  paths; TODO values and failed checks raise manual_review; overrides
  propagate to every downstream line
- Mixed currencies converted via currency.yaml
- SQLite storage: quote revisions, override log, actuals, library hash
- Excel and PDF quote breakdown, Streamlit UI, CLI quote/regress/app
- Reference-set regression against actual cost (±tolerance)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F5coqS3eD35hPcxKNXwKTB
</commit_message>
<xml_diff>
--- a/templates/referans_teklifler.xlsx
+++ b/templates/referans_teklifler.xlsx
@@ -207,7 +207,7 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Prepreg / malzeme (serbest metin veya kütüphane id)</t>
+        <t>Ana prepreg: kütüphane id (örn. PP_CF_UD_120); yoksa serbest metin</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -273,110 +273,140 @@
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>Mühendis değerlendirmesi</t>
+        <t>Kalıp torbalama alanı (flanş, run-off dahil)
+Birim: m2</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>Kalıp malzeme sınıfı</t>
+        <t>Kalıp torbalama çevresi
+Birim: m</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
+        <t>Kalıbın autoclave taban izi, X
+Birim: mm</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Kalıbın autoclave taban izi, Y
+Birim: mm</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Siparişin ilk parçasının kümülatif sıra no (yeni iş = 1)
+Birim: adet</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Mühendis değerlendirmesi</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>Kalıp malzeme sınıfı</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
         <t>Ters açı çözümü</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t>Bu satırdaki tüm tutarların para birimi
 Zorunlu</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: malzeme (fire dahil)
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: sarf
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: işçilik süresi
 Birim: adam-saat/adet</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: işçilik tutarı
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: autoclave payı
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: kalıp + master model (NRE, toplam)
 Birim: para birimi</t>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
+    <comment ref="AI1" authorId="0" shapeId="0">
       <text>
         <t>Teklif: birim satış fiyatı (NRE hariç)
 Birim: para birimi/adet
 Zorunlu</t>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
+    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: malzeme
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
+    <comment ref="AK1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: sarf
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
+    <comment ref="AL1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: işçilik süresi
 Birim: adam-saat/adet</t>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AM1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: işçilik tutarı
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0" shapeId="0">
+    <comment ref="AN1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: kalıp + master model (toplam)
 Birim: para birimi</t>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
+    <comment ref="AO1" authorId="0" shapeId="0">
       <text>
         <t>Gerçekleşen: birim maliyet (NRE hariç)
 Birim: para birimi/adet</t>
       </text>
     </comment>
-    <comment ref="AK1" authorId="0" shapeId="0">
+    <comment ref="AP1" authorId="0" shapeId="0">
       <text>
         <t>Teklif kazanıldı mı</t>
       </text>
     </comment>
-    <comment ref="AL1" authorId="0" shapeId="0">
+    <comment ref="AQ1" authorId="0" shapeId="0">
       <text>
         <t>Serbest not</t>
       </text>
@@ -674,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL2001"/>
+  <dimension ref="A1:AQ2001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -696,25 +726,30 @@
     <col width="19" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="32" customWidth="1" min="24" max="24"/>
-    <col width="32" customWidth="1" min="25" max="25"/>
-    <col width="32" customWidth="1" min="26" max="26"/>
-    <col width="32" customWidth="1" min="27" max="27"/>
-    <col width="32" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="17" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
     <col width="32" customWidth="1" min="29" max="29"/>
     <col width="32" customWidth="1" min="30" max="30"/>
     <col width="32" customWidth="1" min="31" max="31"/>
-    <col width="31" customWidth="1" min="32" max="32"/>
+    <col width="32" customWidth="1" min="32" max="32"/>
     <col width="32" customWidth="1" min="33" max="33"/>
     <col width="32" customWidth="1" min="34" max="34"/>
-    <col width="31" customWidth="1" min="35" max="35"/>
+    <col width="32" customWidth="1" min="35" max="35"/>
     <col width="32" customWidth="1" min="36" max="36"/>
-    <col width="14" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
+    <col width="31" customWidth="1" min="37" max="37"/>
+    <col width="32" customWidth="1" min="38" max="38"/>
+    <col width="32" customWidth="1" min="39" max="39"/>
+    <col width="31" customWidth="1" min="40" max="40"/>
+    <col width="32" customWidth="1" min="41" max="41"/>
+    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="14" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -815,95 +850,120 @@
       </c>
       <c r="T1" s="2" t="inlineStr">
         <is>
+          <t>kalip_alani [m2]</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>kalip_cevresi [m]</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>kalip_zarf_x [mm]</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>kalip_zarf_y [mm]</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>ilk_parca_sira_no [adet]</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
           <t>karmasiklik</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>kalip_cinsi</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>ters_aci_cozumu</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>para_birimi</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>teklif_malzeme [para birimi/adet]</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>teklif_sarf [para birimi/adet]</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>teklif_iscilik_saat [adam-saat/adet]</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>teklif_iscilik [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>teklif_autoclave [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>teklif_kalip_nre [para birimi]</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>teklif_birim_fiyat [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>fiili_malzeme [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>fiili_sarf [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>fiili_iscilik_saat [adam-saat/adet]</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>fiili_iscilik [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>fiili_kalip_nre [para birimi]</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>fiili_birim_maliyet [para birimi/adet]</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>kazanildi</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>notlar</t>
         </is>
@@ -6910,7 +6970,7 @@
       <c r="B2001" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="31">
+  <dataValidations count="36">
     <dataValidation sqref="B2:B2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Tarih girin (GG.AA.YYYY)." type="date" operator="greaterThan">
       <formula1>1</formula1>
     </dataValidation>
@@ -6950,32 +7010,32 @@
     <dataValidation sqref="S2:S2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="0 veya daha büyük bir tam sayı girin." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
+    <dataValidation sqref="T2:T2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="0 veya daha büyük bir tam sayı girin." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
       <formula1>Listeler!$C$2:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
+    <dataValidation sqref="Z2:Z2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
       <formula1>Listeler!$E$2:$E$8</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
+    <dataValidation sqref="AA2:AA2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
       <formula1>Listeler!$G$2:$G$8</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
+    <dataValidation sqref="AB2:AB2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
       <formula1>Listeler!$I$2:$I$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="X2:X2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
-      <formula1>-1000000000</formula1>
-    </dataValidation>
-    <dataValidation sqref="Y2:Y2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
-      <formula1>-1000000000</formula1>
-    </dataValidation>
-    <dataValidation sqref="Z2:Z2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
-      <formula1>-1000000000</formula1>
-    </dataValidation>
-    <dataValidation sqref="AA2:AA2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
-      <formula1>-1000000000</formula1>
-    </dataValidation>
-    <dataValidation sqref="AB2:AB2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
-      <formula1>-1000000000</formula1>
     </dataValidation>
     <dataValidation sqref="AC2:AC2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
@@ -7001,7 +7061,22 @@
     <dataValidation sqref="AJ2:AJ2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
       <formula1>-1000000000</formula1>
     </dataValidation>
-    <dataValidation sqref="AK2:AK2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
+    <dataValidation sqref="AK2:AK2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="AL2:AL2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="AM2:AM2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="AN2:AN2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="AO2:AO2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Sayı girin (ondalık ayırıcı Excel ayarınıza göre)." type="decimal" operator="greaterThanOrEqual">
+      <formula1>-1000000000</formula1>
+    </dataValidation>
+    <dataValidation sqref="AP2:AP2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen listeden seçin (Listeler sayfası)." type="list">
       <formula1>Listeler!$K$2:$K$3</formula1>
     </dataValidation>
   </dataValidations>
@@ -7016,7 +7091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7272,7 +7347,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prepreg / malzeme (serbest metin veya kütüphane id)</t>
+          <t>Ana prepreg: kütüphane id (örn. PP_CF_UD_120); yoksa serbest metin</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -7531,122 +7606,118 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>karmasiklik</t>
+          <t>kalip_alani [m2]</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mühendis değerlendirmesi</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>Kalıp torbalama alanı (flanş, run-off dahil)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>liste</t>
+          <t>sayı</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>dusuk, orta, yuksek</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>kalip_cinsi</t>
+          <t>kalip_cevresi [m]</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kalıp malzeme sınıfı</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>Kalıp torbalama çevresi</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>liste</t>
+          <t>sayı</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>tooling_board, gfrp, cfrp, invar, aluminyum, celik, diger</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ters_aci_cozumu</t>
+          <t>kalip_zarf_x [mm]</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ters açı çözümü</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>Kalıbın autoclave taban izi, X</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>liste</t>
+          <t>sayı</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>yok, maca, bolunmus_kalip, mandrel_konik, mandrel_bolunmus, bladder, cozunur_mandrel</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>para_birimi</t>
+          <t>kalip_zarf_y [mm]</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bu satırdaki tüm tutarların para birimi</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>Kalıbın autoclave taban izi, Y</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>liste</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>evet</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>EUR, TRY, USD</t>
-        </is>
-      </c>
+          <t>sayı</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>teklif_malzeme [para birimi/adet]</t>
+          <t>ilk_parca_sira_no [adet]</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Teklif: malzeme (fire dahil)</t>
+          <t>Siparişin ilk parçasının kümülatif sıra no (yeni iş = 1)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>para birimi/adet</t>
+          <t>adet</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>sayı</t>
+          <t>tam sayı</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -7655,113 +7726,117 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>teklif_sarf [para birimi/adet]</t>
+          <t>karmasiklik</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Teklif: sarf</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>para birimi/adet</t>
-        </is>
-      </c>
+          <t>Mühendis değerlendirmesi</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>sayı</t>
+          <t>liste</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>dusuk, orta, yuksek</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>teklif_iscilik_saat [adam-saat/adet]</t>
+          <t>kalip_cinsi</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Teklif: işçilik süresi</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>adam-saat/adet</t>
-        </is>
-      </c>
+          <t>Kalıp malzeme sınıfı</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>sayı</t>
+          <t>liste</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>tooling_board, gfrp, cfrp, invar, aluminyum, celik, diger</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>teklif_iscilik [para birimi/adet]</t>
+          <t>ters_aci_cozumu</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Teklif: işçilik tutarı</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>para birimi/adet</t>
-        </is>
-      </c>
+          <t>Ters açı çözümü</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>sayı</t>
+          <t>liste</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>yok, maca, bolunmus_kalip, mandrel_konik, mandrel_bolunmus, bladder, cozunur_mandrel</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>teklif_autoclave [para birimi/adet]</t>
+          <t>para_birimi</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Teklif: autoclave payı</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>para birimi/adet</t>
-        </is>
-      </c>
+          <t>Bu satırdaki tüm tutarların para birimi</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>sayı</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+          <t>liste</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>EUR, TRY, USD</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>teklif_kalip_nre [para birimi]</t>
+          <t>teklif_malzeme [para birimi/adet]</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Teklif: kalıp + master model (NRE, toplam)</t>
+          <t>Teklif: malzeme (fire dahil)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>para birimi</t>
+          <t>para birimi/adet</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -7775,12 +7850,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>teklif_birim_fiyat [para birimi/adet]</t>
+          <t>teklif_sarf [para birimi/adet]</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Teklif: birim satış fiyatı (NRE hariç)</t>
+          <t>Teklif: sarf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -7793,27 +7868,23 @@
           <t>sayı</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>evet</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>fiili_malzeme [para birimi/adet]</t>
+          <t>teklif_iscilik_saat [adam-saat/adet]</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Gerçekleşen: malzeme</t>
+          <t>Teklif: işçilik süresi</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>para birimi/adet</t>
+          <t>adam-saat/adet</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -7827,12 +7898,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>fiili_sarf [para birimi/adet]</t>
+          <t>teklif_iscilik [para birimi/adet]</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Gerçekleşen: sarf</t>
+          <t>Teklif: işçilik tutarı</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -7851,17 +7922,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>fiili_iscilik_saat [adam-saat/adet]</t>
+          <t>teklif_autoclave [para birimi/adet]</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Gerçekleşen: işçilik süresi</t>
+          <t>Teklif: autoclave payı</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>adam-saat/adet</t>
+          <t>para birimi/adet</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -7875,17 +7946,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>fiili_iscilik [para birimi/adet]</t>
+          <t>teklif_kalip_nre [para birimi]</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Gerçekleşen: işçilik tutarı</t>
+          <t>Teklif: kalıp + master model (NRE, toplam)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>para birimi/adet</t>
+          <t>para birimi</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -7899,17 +7970,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>fiili_kalip_nre [para birimi]</t>
+          <t>teklif_birim_fiyat [para birimi/adet]</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Gerçekleşen: kalıp + master model (toplam)</t>
+          <t>Teklif: birim satış fiyatı (NRE hariç)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>para birimi</t>
+          <t>para birimi/adet</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -7917,18 +7988,22 @@
           <t>sayı</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fiili_birim_maliyet [para birimi/adet]</t>
+          <t>fiili_malzeme [para birimi/adet]</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Gerçekleşen: birim maliyet (NRE hariç)</t>
+          <t>Gerçekleşen: malzeme</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7947,46 +8022,166 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>kazanildi</t>
+          <t>fiili_sarf [para birimi/adet]</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Teklif kazanıldı mı</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>Gerçekleşen: sarf</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>para birimi/adet</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>liste</t>
+          <t>sayı</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>E, H</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>notlar</t>
+          <t>fiili_iscilik_saat [adam-saat/adet]</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Serbest not</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>Gerçekleşen: işçilik süresi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>adam-saat/adet</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>metin</t>
+          <t>sayı</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>fiili_iscilik [para birimi/adet]</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gerçekleşen: işçilik tutarı</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>para birimi/adet</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>sayı</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fiili_kalip_nre [para birimi]</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Gerçekleşen: kalıp + master model (toplam)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>para birimi</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>sayı</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fiili_birim_maliyet [para birimi/adet]</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Gerçekleşen: birim maliyet (NRE hariç)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>para birimi/adet</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>sayı</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>kazanildi</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Teklif kazanıldı mı</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>liste</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>E, H</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>notlar</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Serbest not</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>metin</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>